<commit_message>
feat(paichan/cip): CIP 清洗时序常数(CIP/SIP 时长·分钟 + DHT/CHT·小时)
设备/管线两类清洗对象平级加时序常数,单位写进列名(同 shelf_life_hours):
- ps_cip_equipment: cip_duration_minutes/sip_duration_minutes/dht_hours/cht_hours
- ps_pipeline: cip_duration_minutes/dht_hours/cht_hours
时长用分钟(CIP/SIP 30–120 分整数不丢精度),时效用小时(DHT/CHT);全可空,
留空=不启用。DHT/CHT 落 STN max-lag,驱动 CIP 必须落点。
后端 CRUD/导入/非负整数校验、前端表单(showIf cleaning_mode=cip 联动隐藏)
+清洗参数紧凑列、Excel 模板(I..L / F..H 列 + 数字校验 + 单位说明)全部跟上。
两端 tsc 0;导入实测 PT CIP90/DHT24/CHT72、BIO-2000 +SIP60、免洗设备全 NULL。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/production_scheduling/CIP拓扑导入模板.xlsx
+++ b/docs/production_scheduling/CIP拓扑导入模板.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="108" customWidth="1" min="1" max="1"/>
@@ -548,19 +548,26 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>6) 带 * 的列必填(表头标黄)。下拉填错词会被拒。</t>
+          <t>5b) 清洗时序 + 单位:CIP/SIP 时长用「分钟」,DHT(脏停放=变脏后须几小时内开洗)/ CHT(洁净有效期=洗完几小时内须被用)用「小时」。只对要 CIP 的设备/管线填,免洗的留空。</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>7) 填写顺序:先「站」「房间」→ 再「设备」→ 再「管线」。下游下拉来自上游已录的编码,自动增长。</t>
+          <t>6) 带 * 的列必填(表头标黄)。下拉填错词会被拒。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>7) 填写顺序:先「站」「房间」→ 再「设备」→ 再「管线」。下游下拉来自上游已录的编码,自动增长。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>8) 导入按「设施+编码」upsert:已存在则更新,不存在则新增;重复导入不会建重复。</t>
         </is>
@@ -785,7 +792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -796,7 +803,11 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -842,6 +853,26 @@
       </c>
       <c r="I1" s="4" t="inlineStr">
         <is>
+          <t>CIP时长(分钟)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>SIP时长(分钟)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>DHT(小时)</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>CHT(小时)</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
           <t>备注</t>
         </is>
       </c>
@@ -879,7 +910,17 @@
           <t>CIP-1</t>
         </is>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
         <is>
           <t>组织留空=随房间</t>
         </is>
@@ -918,7 +959,23 @@
           <t>CIP-1</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>CIP后SIP</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -949,9 +1006,13 @@
       </c>
       <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>一次性免CIP,不填站</t>
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr"/>
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>一次性免CIP,站/时长全留空</t>
         </is>
       </c>
     </row>
@@ -988,7 +1049,17 @@
           <t>CIP-1</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>母系统:下面挂多个使用点</t>
         </is>
@@ -1023,7 +1094,11 @@
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>子设备:房间/组织留空→随上级BUF-SYS</t>
         </is>
@@ -1062,10 +1137,20 @@
           <t>CIP-2</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="M7" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="无效值" error="请从下拉中选择有效值" type="list" errorStyle="stop">
       <formula1>=设备类型</formula1>
     </dataValidation>
@@ -1083,6 +1168,9 @@
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="无效值" error="该编码在上游表里还没有,确认无误再继续" promptTitle="提示" prompt="仅清洗方式=CIP 时填,选「站」表里已录的站编码" type="list" errorStyle="warning">
       <formula1>=站编码</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1095,7 +1183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1103,7 +1191,10 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1134,6 +1225,21 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>CIP时长(分钟)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>DHT(小时)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>CHT(小时)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>备注</t>
         </is>
       </c>
@@ -1164,14 +1270,23 @@
           <t>CIP-1</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>示例行</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="无效值" error="该编码在上游表里还没有,确认无误再继续" promptTitle="提示" prompt="选「设备」表里已录的设备编码" type="list" errorStyle="warning">
       <formula1>=设备编码</formula1>
     </dataValidation>
@@ -1180,6 +1295,9 @@
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="无效值" error="该编码在上游表里还没有,确认无误再继续" promptTitle="提示" prompt="选「站」表里已录的站编码" type="list" errorStyle="warning">
       <formula1>=站编码</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>